<commit_message>
[muse-5] VR350 22/10: final comparison + decisions
</commit_message>
<xml_diff>
--- a/2210/comparison_2026-09-17_vs_2026-10-22.xlsx
+++ b/2210/comparison_2026-09-17_vs_2026-10-22.xlsx
@@ -13940,7 +13940,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>needs_confirmation</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -13994,7 +13994,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>needs_confirmation</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>
@@ -14048,7 +14048,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>needs_confirmation</t>
+          <t>confirmed</t>
         </is>
       </c>
     </row>

</xml_diff>